<commit_message>
add missing DH LCOM
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/02_smart_energy/03_evaluation_smart_energy/output_LCOE_comparision_smart-energy.xlsx
+++ b/Spine_Projects/03_output_data/02_smart_energy/03_evaluation_smart_energy/output_LCOE_comparision_smart-energy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\02_smart_energy\03_evaluation_smart_energy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A86C7AC-8A90-41D7-BFBF-2025613FC433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F2A135-2D89-460B-AB49-3EC50C858F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
   <sheets>
     <sheet name="Comparison_scenarios" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="78">
   <si>
     <t>run_name</t>
   </si>
@@ -222,30 +222,6 @@
     <t>2045 base water 10p up</t>
   </si>
   <si>
-    <t>2045 base 02 price 10p down</t>
-  </si>
-  <si>
-    <t>2045 base 02 price 05p down</t>
-  </si>
-  <si>
-    <t>2045 base 02 price 05p up</t>
-  </si>
-  <si>
-    <t>2045 base 02 price 10p up</t>
-  </si>
-  <si>
-    <t>2045 base 02 volume 10p down</t>
-  </si>
-  <si>
-    <t>2045 base 02 volume 05p down</t>
-  </si>
-  <si>
-    <t>2045 base 02 volume 05p up</t>
-  </si>
-  <si>
-    <t>2045 base 02 volume 10p up</t>
-  </si>
-  <si>
     <t>2018 RES</t>
   </si>
   <si>
@@ -259,6 +235,42 @@
   </si>
   <si>
     <t>2045 base PPA price 10p up</t>
+  </si>
+  <si>
+    <t>2045 base O2 price 10p down</t>
+  </si>
+  <si>
+    <t>2045 base O2 price 05p down</t>
+  </si>
+  <si>
+    <t>2045 base O2 price 05p up</t>
+  </si>
+  <si>
+    <t>2045 base O2 price 10p up</t>
+  </si>
+  <si>
+    <t>2045 base O2 volume 10p down</t>
+  </si>
+  <si>
+    <t>2045 base O2 volume 05p down</t>
+  </si>
+  <si>
+    <t>2045 base O2 volume 05p up</t>
+  </si>
+  <si>
+    <t>2045 base O2 volume 10p up</t>
+  </si>
+  <si>
+    <t>2045 base DH price 10p down</t>
+  </si>
+  <si>
+    <t>2045 base DH price 05p down</t>
+  </si>
+  <si>
+    <t>2045 base DH price 05p up</t>
+  </si>
+  <si>
+    <t>2045 base DH price 10p up</t>
   </si>
 </sst>
 </file>
@@ -330,7 +342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -338,6 +350,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -374,13 +387,13 @@
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -403,32 +416,32 @@
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{6128FCF1-7EAF-4DB9-AB65-A4970FF7A7B8}" name="run_name"/>
-    <tableColumn id="9" xr3:uid="{E1E483D4-117D-4835-9726-D5751F56EFA1}" name="scenario" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{57DD338E-2930-40CB-AC06-11C7900CEBAE}" name="LCOE [Euro/MWh]" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{348EEC01-2159-40EC-A41A-F770A2113C35}" name="LCOE [Euro/t]" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{E1A32900-AFFC-4CA8-9A80-FDDFC927842B}" name="total_investment" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{9BDBD209-C39F-484C-957B-614102BD4B2E}" name="annual_costs" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{2F1A07E8-34B3-485A-A334-6B4F6D50721B}" name="annual_rev" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{B1C9F88F-C828-404D-9F5C-8363B244D4A6}" name="energy_production [MWh]" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{DFDA2CA3-CD6F-466B-81A4-84B9B62CB2C6}" name="energy_production [t]" dataDxfId="3">
+    <tableColumn id="9" xr3:uid="{E1E483D4-117D-4835-9726-D5751F56EFA1}" name="scenario" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{57DD338E-2930-40CB-AC06-11C7900CEBAE}" name="LCOE [Euro/MWh]" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{348EEC01-2159-40EC-A41A-F770A2113C35}" name="LCOE [Euro/t]" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{E1A32900-AFFC-4CA8-9A80-FDDFC927842B}" name="total_investment" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{9BDBD209-C39F-484C-957B-614102BD4B2E}" name="annual_costs" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{2F1A07E8-34B3-485A-A334-6B4F6D50721B}" name="annual_rev" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{B1C9F88F-C828-404D-9F5C-8363B244D4A6}" name="energy_production [MWh]" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{DFDA2CA3-CD6F-466B-81A4-84B9B62CB2C6}" name="energy_production [t]" dataDxfId="5">
       <calculatedColumnFormula>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{C340BB5F-846A-40DD-949F-DC14F9BEBD65}" name="pcf_value" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{3E078780-172C-4BE9-A08D-3FB4DFE536AE}" name="Wind Capacity [MW]" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{C5EF052A-9C95-4AB3-9DF1-51A82396DE4F}" name="Size electrolyser [MW]" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{C340BB5F-846A-40DD-949F-DC14F9BEBD65}" name="pcf_value" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{3E078780-172C-4BE9-A08D-3FB4DFE536AE}" name="Wind Capacity [MW]" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{C5EF052A-9C95-4AB3-9DF1-51A82396DE4F}" name="Size electrolyser [MW]" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}" name="Table3" displayName="Table3" ref="A1:D50" totalsRowShown="0">
-  <autoFilter ref="A1:D50" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}" name="Table3" displayName="Table3" ref="A1:D54" totalsRowShown="0">
+  <autoFilter ref="A1:D54" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8869914E-4BE8-401C-AC76-C6570071019E}" name="run_name"/>
     <tableColumn id="4" xr3:uid="{96123E5C-038E-4A38-8295-89FC853EE7AF}" name="type"/>
-    <tableColumn id="2" xr3:uid="{EDC23835-EE0F-4ABC-9DD3-CB899B7BD1E4}" name="LCOE [Euro/MWh]" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{7F3B94FF-49AD-4295-99F8-AE1E37B8E7F6}" name="LCOE [Euro/t]" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{EDC23835-EE0F-4ABC-9DD3-CB899B7BD1E4}" name="LCOE [Euro/MWh]" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{7F3B94FF-49AD-4295-99F8-AE1E37B8E7F6}" name="LCOE [Euro/t]" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1393,7 +1406,7 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C17" s="2">
         <v>194.65979782804271</v>
@@ -1432,7 +1445,7 @@
         <v>2035</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C18" s="2">
         <v>168.97284471743725</v>
@@ -1471,7 +1484,7 @@
         <v>2045</v>
       </c>
       <c r="B19" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2">
         <v>179.98483084041058</v>
@@ -1517,7 +1530,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5837E54A-3435-47A0-958D-D2D4B44DC326}">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.453125" bestFit="1" customWidth="1"/>
@@ -1526,7 +1539,7 @@
     <col min="4" max="4" width="14.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1540,7 +1553,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1557,7 +1570,7 @@
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1571,8 +1584,10 @@
         <v>976.10575871664832</v>
       </c>
       <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G3" s="7"/>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -1586,8 +1601,10 @@
         <v>972.12829863224215</v>
       </c>
       <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G4" s="7"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -1601,8 +1618,10 @@
         <v>965.58701080843218</v>
       </c>
       <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G5" s="7"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -1616,8 +1635,10 @@
         <v>962.88870529324731</v>
       </c>
       <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G6" s="7"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1630,8 +1651,10 @@
       <c r="D7" s="2">
         <v>955.28510095825379</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G7" s="7"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -1644,8 +1667,10 @@
       <c r="D8" s="2">
         <v>961.92033053154273</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G8" s="7"/>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1658,8 +1683,10 @@
       <c r="D9" s="2">
         <v>975.46078723622099</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G9" s="7"/>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1672,8 +1699,10 @@
       <c r="D10" s="2">
         <v>982.35920056445832</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G10" s="7"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1686,8 +1715,10 @@
       <c r="D11" s="2">
         <v>1006.8461109398615</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G11" s="7"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1700,8 +1731,10 @@
       <c r="D12" s="2">
         <v>985.35997551794105</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G12" s="7"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -1714,8 +1747,10 @@
       <c r="D13" s="2">
         <v>979.05982805690769</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G13" s="7"/>
+      <c r="I13" s="2"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -1728,8 +1763,10 @@
       <c r="D14" s="2">
         <v>988.64990382690871</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G14" s="7"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -1742,8 +1779,10 @@
       <c r="D15" s="2">
         <v>962.16213735078668</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G15" s="7"/>
+      <c r="I15" s="2"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -1756,8 +1795,10 @@
       <c r="D16" s="2">
         <v>961.60483105044966</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G16" s="7"/>
+      <c r="I16" s="2"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -1770,8 +1811,10 @@
       <c r="D17" s="2">
         <v>974.76620720828441</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G17" s="7"/>
+      <c r="I17" s="2"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -1784,8 +1827,10 @@
       <c r="D18" s="2">
         <v>1034.6824481906181</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G18" s="7"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -1798,8 +1843,10 @@
       <c r="D19" s="2">
         <v>964.86268787869528</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G19" s="7"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -1812,8 +1859,10 @@
       <c r="D20" s="2">
         <v>966.75469324791572</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G20" s="7"/>
+      <c r="I20" s="2"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -1826,8 +1875,10 @@
       <c r="D21" s="2">
         <v>970.53870398608626</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G21" s="7"/>
+      <c r="I21" s="2"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -1840,8 +1891,10 @@
       <c r="D22" s="2">
         <v>972.43070935513367</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G22" s="7"/>
+      <c r="I22" s="2"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>45</v>
       </c>
@@ -1854,8 +1907,10 @@
       <c r="D23" s="2">
         <v>880.9786559696521</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G23" s="7"/>
+      <c r="I23" s="2"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -1868,8 +1923,10 @@
       <c r="D24" s="2">
         <v>923.08404403070176</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G24" s="7"/>
+      <c r="I24" s="2"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>47</v>
       </c>
@@ -1882,8 +1939,10 @@
       <c r="D25" s="2">
         <v>1045.3573771365486</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G25" s="7"/>
+      <c r="I25" s="2"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -1896,8 +1955,10 @@
       <c r="D26" s="2">
         <v>1119.0405022572638</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G26" s="7"/>
+      <c r="I26" s="2"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>49</v>
       </c>
@@ -1910,8 +1971,10 @@
       <c r="D27" s="2">
         <v>1113.3349164679848</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G27" s="7"/>
+      <c r="I27" s="2"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>50</v>
       </c>
@@ -1924,8 +1987,10 @@
       <c r="D28" s="2">
         <v>1023.5223965290166</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G28" s="7"/>
+      <c r="I28" s="2"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>51</v>
       </c>
@@ -1938,8 +2003,10 @@
       <c r="D29" s="2">
         <v>915.42311870781964</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G29" s="7"/>
+      <c r="I29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>52</v>
       </c>
@@ -1952,8 +2019,10 @@
       <c r="D30" s="2">
         <v>873.90392752176876</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G30" s="7"/>
+      <c r="I30" s="2"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
         <v>53</v>
       </c>
@@ -1966,8 +2035,10 @@
       <c r="D31" s="2">
         <v>953.16216452160177</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G31" s="7"/>
+      <c r="I31" s="2"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
         <v>54</v>
       </c>
@@ -1980,8 +2051,10 @@
       <c r="D32" s="2">
         <v>961.52793194068715</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G32" s="7"/>
+      <c r="I32" s="2"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>55</v>
       </c>
@@ -1994,8 +2067,10 @@
       <c r="D33" s="2">
         <v>975.73485554545823</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G33" s="7"/>
+      <c r="I33" s="2"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="6" t="s">
         <v>56</v>
       </c>
@@ -2008,8 +2083,10 @@
       <c r="D34" s="2">
         <v>982.8042494662227</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G34" s="7"/>
+      <c r="I34" s="2"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
         <v>57</v>
       </c>
@@ -2022,8 +2099,10 @@
       <c r="D35" s="2">
         <v>968.31856599745265</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G35" s="7"/>
+      <c r="I35" s="2"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="s">
         <v>58</v>
       </c>
@@ -2036,8 +2115,10 @@
       <c r="D36" s="2">
         <v>968.48263230716145</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G36" s="7"/>
+      <c r="I36" s="2"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
         <v>59</v>
       </c>
@@ -2050,8 +2131,10 @@
       <c r="D37" s="2">
         <v>968.81076492672003</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G37" s="7"/>
+      <c r="I37" s="2"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
         <v>60</v>
       </c>
@@ -2064,10 +2147,12 @@
       <c r="D38" s="2">
         <v>968.97483123641621</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G38" s="7"/>
+      <c r="I38" s="2"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B39" t="s">
         <v>13</v>
@@ -2078,10 +2163,12 @@
       <c r="D39" s="2">
         <v>994.93640022526245</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G39" s="7"/>
+      <c r="I39" s="2"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B40" t="s">
         <v>13</v>
@@ -2092,10 +2179,12 @@
       <c r="D40" s="2">
         <v>981.79154942106584</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G40" s="7"/>
+      <c r="I40" s="2"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B41" t="s">
         <v>13</v>
@@ -2106,10 +2195,12 @@
       <c r="D41" s="2">
         <v>955.50184781280336</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G41" s="7"/>
+      <c r="I41" s="2"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B42" t="s">
         <v>13</v>
@@ -2120,10 +2211,12 @@
       <c r="D42" s="2">
         <v>942.35699700867542</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G42" s="7"/>
+      <c r="I42" s="2"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B43" t="s">
         <v>13</v>
@@ -2134,10 +2227,12 @@
       <c r="D43" s="2">
         <v>994.93640019999998</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G43" s="7"/>
+      <c r="I43" s="2"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B44" t="s">
         <v>13</v>
@@ -2148,10 +2243,12 @@
       <c r="D44" s="2">
         <v>981.79154942106584</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G44" s="7"/>
+      <c r="I44" s="2"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B45" t="s">
         <v>13</v>
@@ -2162,10 +2259,12 @@
       <c r="D45" s="2">
         <v>955.50184781280336</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G45" s="7"/>
+      <c r="I45" s="2"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B46" t="s">
         <v>13</v>
@@ -2176,10 +2275,12 @@
       <c r="D46" s="2">
         <v>942.35699700867542</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G46" s="7"/>
+      <c r="I46" s="2"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B47" t="s">
         <v>13</v>
@@ -2190,10 +2291,12 @@
       <c r="D47" s="2">
         <v>966.77345781271913</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G47" s="7"/>
+      <c r="I47" s="2"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B48" t="s">
         <v>13</v>
@@ -2204,10 +2307,12 @@
       <c r="D48" s="2">
         <v>967.71252617883192</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G48" s="7"/>
+      <c r="I48" s="2"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B49" t="s">
         <v>13</v>
@@ -2218,10 +2323,12 @@
       <c r="D49" s="2">
         <v>969.5442161176602</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G49" s="7"/>
+      <c r="I49" s="2"/>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B50" t="s">
         <v>13</v>
@@ -2232,6 +2339,72 @@
       <c r="D50" s="2">
         <v>970.46445241074798</v>
       </c>
+      <c r="G50" s="7"/>
+      <c r="I50" s="2"/>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>74</v>
+      </c>
+      <c r="B51" t="s">
+        <v>13</v>
+      </c>
+      <c r="C51" s="2">
+        <v>175.54369062241958</v>
+      </c>
+      <c r="D51" s="2">
+        <v>970.36651205170813</v>
+      </c>
+      <c r="G51" s="7"/>
+      <c r="I51" s="2"/>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>75</v>
+      </c>
+      <c r="B52" t="s">
+        <v>13</v>
+      </c>
+      <c r="C52" s="2">
+        <v>175.38812960821986</v>
+      </c>
+      <c r="D52" s="2">
+        <v>969.50660533432631</v>
+      </c>
+      <c r="G52" s="7"/>
+      <c r="I52" s="2"/>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>76</v>
+      </c>
+      <c r="B53" t="s">
+        <v>13</v>
+      </c>
+      <c r="C53" s="2">
+        <v>175.07700757982079</v>
+      </c>
+      <c r="D53" s="2">
+        <v>967.78679189956483</v>
+      </c>
+      <c r="G53" s="7"/>
+      <c r="I53" s="2"/>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>77</v>
+      </c>
+      <c r="B54" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" s="2">
+        <v>174.92144656562206</v>
+      </c>
+      <c r="D54" s="2">
+        <v>966.92688518218847</v>
+      </c>
+      <c r="G54" s="7"/>
+      <c r="I54" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>